<commit_message>
Update manuscript figures and add failure-analysis visualizations
</commit_message>
<xml_diff>
--- a/manuscript/manuscript_narrative/original_layout/brief_communication/figures/Source_Data_Fig2.xlsx
+++ b/manuscript/manuscript_narrative/original_layout/brief_communication/figures/Source_Data_Fig2.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2a" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2b" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2c" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig2d" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -775,13 +776,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>benchmark</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -791,186 +792,209 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>steps_with_record</t>
+          <t>Single run</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>steps</t>
+          <t>Majority of 3</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>Majority of 12</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>At least 1 of 3 correct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>answer_vote_of_3</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>replicate_groups</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Command</t>
+          <t>BixBench-Verified-50</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>custom code</t>
+          <t>Galaxy</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55380</v>
+        <v>87.67</v>
       </c>
       <c r="D2" t="n">
-        <v>55380</v>
+        <v>88</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>92</v>
+      </c>
+      <c r="F2" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Command</t>
+          <t>BixBench-Verified-50</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Galaxy</t>
+          <t>custom code</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>36078</v>
+        <v>87.17</v>
       </c>
       <c r="D3" t="n">
-        <v>37498</v>
+        <v>89.5</v>
       </c>
       <c r="E3" t="n">
-        <v>96.21313136700624</v>
+        <v>90</v>
+      </c>
+      <c r="F3" t="n">
+        <v>91</v>
+      </c>
+      <c r="G3" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tool and version</t>
+          <t>CompBioBench</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>custom code</t>
+          <t>Galaxy</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="D4" t="n">
-        <v>55380</v>
+        <v>87.25</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>91</v>
+      </c>
+      <c r="F4" t="n">
+        <v>94.25</v>
+      </c>
+      <c r="G4" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="H4" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tool and version</t>
+          <t>CompBioBench</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Galaxy</t>
+          <t>custom code</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>37498</v>
+        <v>86.67</v>
       </c>
       <c r="D5" t="n">
-        <v>37498</v>
+        <v>89</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>89</v>
+      </c>
+      <c r="F5" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="G5" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Parameters</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>custom code</t>
+          <t>Galaxy</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="D6" t="n">
-        <v>55380</v>
+        <v>80</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>80</v>
+      </c>
+      <c r="F6" t="n">
+        <v>85</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Parameters</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Galaxy</t>
+          <t>custom code</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>37498</v>
+        <v>74.17</v>
       </c>
       <c r="D7" t="n">
-        <v>37498</v>
+        <v>72.5</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Output datasets</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>custom code</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>55380</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Output datasets</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Galaxy</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>37498</v>
-      </c>
-      <c r="D9" t="n">
-        <v>37498</v>
-      </c>
-      <c r="E9" t="n">
-        <v>100</v>
+        <v>70</v>
+      </c>
+      <c r="F7" t="n">
+        <v>85</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -984,127 +1008,280 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>stage</t>
+          <t>element</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>galaxy_tokens_millions</t>
+          <t>galaxy</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>custom_code_tokens_millions</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>galaxy_over_custom_code</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>galaxy_runs_correct_pct</t>
+          <t>custom_code</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>July: Round 1 in place: shorter skills, prompt guidance</t>
+          <t>Tool and version</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>featurewise_correlation 0.1.0+galaxy3 (Tool Shed identifier)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Inline Python script; pandas, NumPy and SciPy installed with unpinned pip</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Parameters</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fields: method = spearman; transform_b = negate; min_pairs = 3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Written in the code; essentiality taken as −ρ when ranking</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Inputs and
+outputs</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2 input and 2 output datasets, linked by identifier in the history</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Inputs named in the code; results printed to the log only</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Job state "ok", exit code 0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Exit code per command (5 of 21 analysis commands failed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CDKN1A (accepted)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CDKN1A (accepted)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>galaxy_over_custom_code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ci95_low</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ci95_high</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>galaxy_runs_correct_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>galaxy_tokens_millions</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>custom_code_tokens_millions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Round 1</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>148.913163</v>
+        <v>5.479528789913112</v>
       </c>
       <c r="C2" t="n">
-        <v>27.17627166666667</v>
+        <v>4.1667</v>
       </c>
       <c r="D2" t="n">
-        <v>5.479528789913112</v>
+        <v>7.2571</v>
       </c>
       <c r="E2" t="n">
         <v>92.66666666666666</v>
       </c>
+      <c r="F2" t="n">
+        <v>148.913163</v>
+      </c>
+      <c r="G2" t="n">
+        <v>27.17627166666667</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>July: Round 2: submit, wait and check in one MCP call</t>
+          <t>Round 2</t>
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2.807705901314365</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.1117</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.8022</v>
+      </c>
+      <c r="E3" t="n">
+        <v>91.33333333333333</v>
+      </c>
+      <c r="F3" t="n">
         <v>66.64810133333333</v>
       </c>
-      <c r="C3" t="n">
+      <c r="G3" t="n">
         <v>23.737565</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2.807705901314365</v>
-      </c>
-      <c r="E3" t="n">
-        <v>91.33333333333331</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>October: Archived runs (round 2 in place)</t>
+          <t>Round 2 (main runs)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>122.414454</v>
+        <v>3.446950135954488</v>
       </c>
       <c r="C4" t="n">
-        <v>35.51384533333334</v>
+        <v>1.6524</v>
       </c>
       <c r="D4" t="n">
-        <v>3.446950135954488</v>
+        <v>7.1471</v>
       </c>
       <c r="E4" t="n">
         <v>90.66666666666666</v>
       </c>
+      <c r="F4" t="n">
+        <v>122.414454</v>
+      </c>
+      <c r="G4" t="n">
+        <v>35.51384533333334</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>October: Round 3: compact replies, templates (1 replicate)</t>
+          <t>Round 3 (1 replicate)</t>
         </is>
       </c>
       <c r="B5" t="n">
+        <v>2.419729099832013</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
         <v>85.933885</v>
       </c>
-      <c r="C5" t="n">
+      <c r="G5" t="n">
         <v>35.51384533333334</v>
       </c>
-      <c r="D5" t="n">
-        <v>2.419729099832013</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>October: Round 3 plus longer waits between requests</t>
+          <t>Round 3 + longer waits</t>
         </is>
       </c>
       <c r="B6" t="n">
+        <v>1.530369864387914</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.7714</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3.0076</v>
+      </c>
+      <c r="E6" t="n">
+        <v>91.33333333333333</v>
+      </c>
+      <c r="F6" t="n">
         <v>54.34931866666666</v>
       </c>
-      <c r="C6" t="n">
+      <c r="G6" t="n">
         <v>35.51384533333334</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1.530369864387914</v>
-      </c>
-      <c r="E6" t="n">
-        <v>91.33333333333331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>